<commit_message>
Executed on 23 July
</commit_message>
<xml_diff>
--- a/Encollect_Web_DBS_P3/Cypress/fixtures/ENCollectSecondaryAllocationCollectionStaff_Customerlevel.xlsx
+++ b/Encollect_Web_DBS_P3/Cypress/fixtures/ENCollectSecondaryAllocationCollectionStaff_Customerlevel.xlsx
@@ -416,7 +416,13 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="str">
-        <v>10008932</v>
+        <v>41174</v>
+      </c>
+      <c r="B2" s="1" t="str">
+        <v>1660</v>
+      </c>
+      <c r="C2" s="1" t="str">
+        <v>2025-20-11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>